<commit_message>
refactor: reorganize media assets into a dedicated directory and remove redundant project documentation
</commit_message>
<xml_diff>
--- a/voting_form.xlsx
+++ b/voting_form.xlsx
@@ -1650,7 +1650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC20"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.19921875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -2160,37 +2160,27 @@
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
-          <t>select_one party_list</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>party_vote</t>
+          <t>religion_other</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cast Your Vote (EVM)</t>
+          <t>Other Religion (Please specify)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>अपना वोट डालें (ईवीएम)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Press the blue button next to the party of your choice to cast your vote.</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>अपना वोट डालने के लिए अपनी पसंद की पार्टी के आगे वाले नीले बटन को दबाएं।</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>custom-evm_vote</t>
+          <t>अन्य धर्म (कृपया निर्दिष्ट करें)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>${religion} = 'other'</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2202,68 +2192,109 @@
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one party_list</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>remarks</t>
+          <t>party_vote</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Respondent Remarks</t>
+          <t>Cast Your Vote (EVM)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>उत्तरदाता की टिप्पणी</t>
+          <t>अपना वोट डालें (ईवीएम)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Press the blue button next to the party of your choice to cast your vote.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>अपना वोट डालने के लिए अपनी पसंद की पार्टी के आगे वाले नीले बटन को दबाएं।</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>custom-evm_vote</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Respondent Remarks</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>उत्तरदाता की टिप्पणी</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>geopoint</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>GPS Location</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>जीपीएस स्थान</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Capture the current GPS coordinates.</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>वर्तमान जीपीएस निर्देशांक कैप्चर करें।</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1"/>
@@ -3392,7 +3423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA41"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.19921875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="15.3984375" customWidth="1" min="1" max="1"/>
@@ -4434,15 +4465,249 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
-    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>district_list</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NDD</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>North Delhi</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>उत्तर दिल्ली</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>DL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>district_list</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Nagpur</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>नागपुर</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>district_list</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>गोरखपुर</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>constituency_list</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>CC_C</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Chandni Chowk</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>चांदनी चौक</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>NDD</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>constituency_list</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>NOD_C</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>North Delhi</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>उत्तर दिल्ली</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>NDD</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>constituency_list</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>NGP_C</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Nagpur</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>नागपुर</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>constituency_list</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>RT_C</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Ramtek</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>रामटेक</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>constituency_list</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GKP_C</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>गोरखपुर</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>constituency_list</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BG_C</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Bansgaon</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>बांसगांव</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+    </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
     <row r="53" ht="15.75" customHeight="1"/>

</xml_diff>